<commit_message>
List the people and their roles under the timeline.
Jacky (project lead, software), Navy (design: UI/UX, characters and
content, store artwork) and Neo (native app shell and store release)
now appear in a table under the weekly timeline and in roadmap.md. The
software sheet names Jacky instead of 我方軟件.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,12 @@
       <name val="Microsoft JhengHei"/>
       <b val="1"/>
       <color rgb="0017202B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="0017202B"/>
       <sz val="14"/>
     </font>
   </fonts>
@@ -83,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -104,6 +110,50 @@
       <bottom style="thin">
         <color rgb="00C9CED6"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9CED6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CED6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CED6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CED6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CED6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9CED6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9CED6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9CED6"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -142,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -165,14 +215,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -538,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1146,12 +1199,111 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>參與人</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>負責</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="10" t="n"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>項目負責人；軟件開發</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>統籌時間表，對接玩具廠、電路板供應商和客戶；開發網頁、後台、語音系統、韌體、Tool call 和 RAG，部署三套系統；負責測試和 UAT</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="10" t="n"/>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Navy</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>三套 UI／UX 設計；角色和內容（人設、說話風格、開場白、聲線、角色圖）；App 圖示、啟動畫面和商店截圖</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="10" t="n"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>App 殼</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；和 Jacky 定網頁對接方式；出測試版，提交蘋果和 Google 審核並上架</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="10" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="12">
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="D28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -1176,16 +1328,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>軟件開發與測試：網頁、App、Tool call、RAG、後台、測試、UAT</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>網頁 App 包在原生殼裡，1/15 上架快活和政協青年聯會兩個 App（AI Buddy 隨玩具延後）。殼由 Neo 負責；設計、角色和 App 圖由 Navy 負責；「我方軟件」是網頁、後台、語音系統和韌體。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>網頁 App 包在原生殼裡，1/15 上架快活和政協青年聯會兩個 App（AI Buddy 隨玩具延後）。殼由 Neo 負責；設計、角色和 App 圖由 Navy 負責；網頁、後台、語音系統和韌體由 Jacky 負責。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1374,7 @@
       </c>
     </row>
     <row r="5" ht="56" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -1232,7 +1384,7 @@
           <t>W1–W2</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>10/23</t>
         </is>
@@ -1254,13 +1406,13 @@
       </c>
     </row>
     <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="12" t="n"/>
+      <c r="A6" s="15" t="n"/>
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>W2–W4</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
@@ -1281,21 +1433,21 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="56" customHeight="1">
-      <c r="A7" s="12" t="n"/>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="15" t="n"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>W2–W5</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>11/13</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Navy；我方軟件放進系統</t>
+          <t>Navy；Jacky 放進系統</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1310,13 +1462,13 @@
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="13" t="n"/>
+      <c r="A8" s="16" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>W6–W7</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
@@ -1338,7 +1490,7 @@
       </c>
     </row>
     <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>網頁</t>
         </is>
@@ -1348,14 +1500,14 @@
           <t>W1–W3</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>10/30</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1370,20 +1522,20 @@
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="12" t="n"/>
+      <c r="A10" s="15" t="n"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>W3–W4</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1398,20 +1550,20 @@
       </c>
     </row>
     <row r="11" ht="56" customHeight="1">
-      <c r="A11" s="12" t="n"/>
+      <c r="A11" s="15" t="n"/>
       <c r="B11" s="4" t="inlineStr">
         <is>
           <t>W4–W6</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1426,20 +1578,20 @@
       </c>
     </row>
     <row r="12" ht="56" customHeight="1">
-      <c r="A12" s="13" t="n"/>
+      <c r="A12" s="16" t="n"/>
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1454,7 +1606,7 @@
       </c>
     </row>
     <row r="13" ht="56" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>App 殼與上架</t>
         </is>
@@ -1464,14 +1616,14 @@
           <t>W1–W2</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>10/23</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Neo、我方軟件</t>
+          <t>Neo、Jacky</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1486,13 +1638,13 @@
       </c>
     </row>
     <row r="14" ht="56" customHeight="1">
-      <c r="A14" s="12" t="n"/>
+      <c r="A14" s="15" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>W3–W6</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
@@ -1514,13 +1666,13 @@
       </c>
     </row>
     <row r="15" ht="56" customHeight="1">
-      <c r="A15" s="12" t="n"/>
+      <c r="A15" s="15" t="n"/>
       <c r="B15" s="4" t="inlineStr">
         <is>
           <t>W8–W9</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>12/11</t>
         </is>
@@ -1542,13 +1694,13 @@
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="13" t="n"/>
+      <c r="A16" s="16" t="n"/>
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>1/15</t>
         </is>
@@ -1570,7 +1722,7 @@
       </c>
     </row>
     <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Tool call</t>
         </is>
@@ -1580,14 +1732,14 @@
           <t>W2–W3</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>10/30</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1602,20 +1754,20 @@
       </c>
     </row>
     <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="13" t="n"/>
+      <c r="A18" s="16" t="n"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>W4–W6</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1629,8 +1781,8 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="56" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>RAG 知識庫（快活）</t>
         </is>
@@ -1640,14 +1792,14 @@
           <t>W4</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>馬會提供資料；我方軟件</t>
+          <t>馬會提供資料；Jacky</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1662,20 +1814,20 @@
       </c>
     </row>
     <row r="20" ht="56" customHeight="1">
-      <c r="A20" s="12" t="n"/>
+      <c r="A20" s="15" t="n"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>W5–W8</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>12/4</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1689,21 +1841,21 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="56" customHeight="1">
-      <c r="A21" s="13" t="n"/>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="16" t="n"/>
       <c r="B21" s="4" t="inlineStr">
         <is>
           <t>W9–W11</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>12/25</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>馬會審核；我方軟件修改</t>
+          <t>馬會審核；Jacky 修改</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1718,7 +1870,7 @@
       </c>
     </row>
     <row r="22" ht="56" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>後台管理</t>
         </is>
@@ -1728,14 +1880,14 @@
           <t>W3–W6</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -1750,20 +1902,20 @@
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="13" t="n"/>
+      <c r="A23" s="16" t="n"/>
       <c r="B23" s="4" t="inlineStr">
         <is>
           <t>W6–W8</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>12/4</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -1778,7 +1930,7 @@
       </c>
     </row>
     <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>測試</t>
         </is>
@@ -1788,14 +1940,14 @@
           <t>W4–W7</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>我方全體</t>
+          <t>全體</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1810,20 +1962,20 @@
       </c>
     </row>
     <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="13" t="n"/>
+      <c r="A25" s="16" t="n"/>
       <c r="B25" s="4" t="inlineStr">
         <is>
           <t>W7–W8</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>12/4</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1838,7 +1990,7 @@
       </c>
     </row>
     <row r="26" ht="56" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -1848,14 +2000,14 @@
           <t>W9–W10</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>12/18</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>馬會、政協青年聯會；我方</t>
+          <t>馬會、政協青年聯會；Jacky</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -1870,20 +2022,20 @@
       </c>
     </row>
     <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="13" t="n"/>
+      <c r="A27" s="16" t="n"/>
       <c r="B27" s="4" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>我方軟件</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Send Navy's app images to Jacky, and Jacky's interface spec to Neo.
The app screens are web pages Jacky builds, so Navy's page designs,
cut assets and store artwork go to Jacky. Neo builds the native shell
from the interface parameters Jacky hands over in W1–W2 (the existing
原生App殼接口文檔). Roles in the people table say the same.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>審 3D 圖；決定電路板改不改；和 Neo 定好 App 殼和網頁的對接方式；Navy 出 UI／UX 設計方向</t>
+          <t>審 3D 圖；決定電路板改不改；Jacky 把 App 接口參數交給 Neo；Navy 出 UI／UX 設計方向</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>2 個工作天內回覆 3D 圖意見；改不改板有書面結論；對接清單由 Neo 確認；設計方向交客戶</t>
+          <t>2 個工作天內回覆 3D 圖意見；改不改板有書面結論；接口參數 Neo 確認可以開發；設計方向交客戶</t>
         </is>
       </c>
     </row>
@@ -1241,14 +1241,14 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>統籌時間表，對接玩具廠、電路板供應商和客戶；開發網頁、後台、語音系統、韌體、Tool call 和 RAG，部署三套系統；負責測試和 UAT</t>
+          <t>統籌時間表，對接玩具廠、電路板供應商和客戶；開發網頁（把 Navy 的設計圖做進 App 畫面）、後台、語音系統、韌體、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；負責測試和 UAT</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="10" t="n"/>
     </row>
-    <row r="27" ht="24" customHeight="1">
+    <row r="27" ht="40" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Navy</t>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>三套 UI／UX 設計；角色和內容（人設、說話風格、開場白、聲線、角色圖）；App 圖示、啟動畫面和商店截圖</t>
+          <t>三套 UI／UX 設計；角色和內容（人設、說話風格、開場白、聲線、角色圖）；App 設計圖、圖示、啟動畫面和商店截圖，全部交給 Jacky</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；和 Jacky 定網頁對接方式；出測試版，提交蘋果和 Google 審核並上架</t>
+          <t>按 Jacky 給的接口參數，開發 iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；出測試版，提交蘋果和 Google 審核並上架</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Navy → Jacky</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>配網、綁定、首頁、對話、記憶、設定、語言等頁面的設計稿可以直接開發；政協青年聯會版只換顏色、logo、插圖；客戶確認</t>
+          <t>配網、綁定、首頁、對話、記憶、設定、語言等頁面的設計稿和切圖交給 Jacky，可以直接做進網頁；政協青年聯會版只換顏色、logo、插圖；客戶確認</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Navy → Neo</t>
+          <t>Navy → Jacky</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>兩個 App 的圖示、啟動畫面、商店截圖和宣傳圖，按蘋果和 Google 的尺寸交給 Neo</t>
+          <t>兩個 App 的圖示、啟動畫面、商店截圖和宣傳圖，按蘋果和 Google 的尺寸交給 Jacky</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="56" customHeight="1">
+    <row r="13" ht="72" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
           <t>App 殼與上架</t>
@@ -1623,17 +1623,17 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Neo、Jacky</t>
+          <t>Jacky → Neo</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>網頁和殼的對接方案</t>
+          <t>Jacky 交 App 接口參數給 Neo</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>對接清單（藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結）逐項寫明介面和錯誤，Neo 書面確認；兩個 App 的名稱、圖示、bundle id 定好</t>
+          <t>接口文件交給 Neo：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明參數、回傳和錯誤；Neo 確認看得懂、可以開發；兩個 App 的名稱、圖示、bundle id 定好</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>殼開發、測試版</t>
+          <t>按接口參數開發殼、出測試版</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">

</xml_diff>

<commit_message>
State that the web is built once with three skins.
The user confirmed one web codebase with three brand skins switched by
configuration; brand differences in function are feature flags, not
separate pages. The first web step, the 快活/政協 step, Jacky's role and
the decision log now say so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>統籌時間表，對接玩具廠、電路板供應商和客戶；開發網頁（把 Navy 的設計圖做進 App 畫面）、後台、語音系統、韌體、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；負責測試和 UAT</t>
+          <t>統籌時間表，對接玩具廠、電路板供應商和客戶；統一開發一套網頁、三套外觀（把 Navy 的設計圖做進 App 畫面）、後台、語音系統、韌體、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；負責測試和 UAT</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
@@ -1337,7 +1337,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>網頁 App 包在原生殼裡，1/15 上架快活和政協青年聯會兩個 App（AI Buddy 隨玩具延後）。殼由 Neo 負責；設計、角色和 App 圖由 Navy 負責；網頁、後台、語音系統和韌體由 Jacky 負責。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
+          <t>網頁統一開發一套，三個品牌是三套外觀，包在原生殼裡；1/15 上架快活和政協青年聯會兩個 App（AI Buddy 隨玩具延後）。殼由 Neo 負責；設計、角色和 App 圖由 Navy 負責；網頁、後台、語音系統和韌體由 Jacky 負責。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
+    <row r="9" ht="88" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
           <t>網頁</t>
@@ -1512,12 +1512,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>共用基礎：品牌主題、App 內登入、刪除帳號</t>
+          <t>統一開發一套網頁，三套外觀；App 內登入、刪除帳號</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>快活、政協青年聯會的顏色、logo、文案顯示正確，畫面不閃；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
+          <t>同一套程式碼按設定切換三套外觀（快活、政協青年聯會、AI Buddy）：顏色、字體、logo、圖示、文案；共用元件裡沒有寫死的品牌；加一套外觀不用改程式；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
         </is>
       </c>
     </row>
@@ -1568,12 +1568,12 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>快活專屬功能；政協青年聯會換主題</t>
+          <t>快活的功能開關；政協青年聯會套用外觀</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）；政協青年聯會版：共用快活的成人版流程，只換顏色、logo、文案和角色</t>
+          <t>同一套網頁裡打開快活的功能：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）；政協青年聯會版用同一套成人版流程，只換外觀和角色</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Navy responsible for the IP designs too.
Navy designs the 政協青年聯會 plush (front, side, back, size, colour,
materials) for the factory by 10/16, and reviews every sample round's
appearance against the design until the 11/13 sign-off. W1 and W3 of the
weekly table and Navy's role say so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -654,7 +654,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="72" customHeight="1">
+    <row r="5" ht="88" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>W1</t>
@@ -682,7 +682,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>定下全部 IP 造型交玩具廠（目前只交了馬會）；交機芯規格；向電路板供應商詢價、追加樣板</t>
+          <t>Navy 完成政協青年聯會版的 IP 造型設計，交玩具廠（馬會的已交）；交機芯規格；向電路板供應商詢價、追加樣板</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>裝板實測，給修改意見；電路板定案；App 登入和品牌主題</t>
+          <t>裝板實測，給修改意見；Navy 給外觀意見；電路板定案；App 登入和品牌主題</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1248,7 +1248,7 @@
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="10" t="n"/>
     </row>
-    <row r="27" ht="40" customHeight="1">
+    <row r="27" ht="56" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Navy</t>
@@ -1257,12 +1257,12 @@
       <c r="B27" s="10" t="n"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>設計</t>
+          <t>設計（IP 造型、UI／UX、角色）</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>三套 UI／UX 設計；角色和內容（人設、說話風格、開場白、聲線、角色圖）；App 設計圖、圖示、啟動畫面和商店截圖，全部交給 Jacky</t>
+          <t>IP 造型設計（政協青年聯會版等），跟進打樣外觀到簽樣；三套 UI／UX 設計；角色和內容（人設、說話風格、開場白、聲線、角色圖）；App 設計圖、圖示、啟動畫面和商店截圖，全部交給 Jacky</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -1316,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1381,375 +1381,371 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>W1–W2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Navy → 玩具廠</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>三套 UI／UX 設計方向</t>
+          <t>IP 造型設計</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>快活、政協青年聯會、AI Buddy 各一份設計規範（顏色、字體、圖示、按鈕）和主要頁面線框；快活和政協青年聯會的方向經客戶確認（AI Buddy 可以晚一點）</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
+          <t>政協青年聯會版的造型圖（正、側、背面，尺寸，顏色，材質建議）交給玩具廠；馬會兩款已交；AI Buddy 造型可以延後</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="15" t="n"/>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>W2–W4</t>
+          <t>W3–W5</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>11/6</t>
+          <t>11/13</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Navy → Jacky</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>快活、政協青年聯會的頁面設計稿</t>
+          <t>跟進打樣外觀</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>配網、綁定、首頁、對話、記憶、設定、語言等頁面的設計稿和切圖交給 Jacky，可以直接做進網頁；政協青年聯會版只換顏色、logo、插圖；客戶確認</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+          <t>每一輪樣品都對照造型圖給外觀修改意見；11/13 簽樣時外觀和設計一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="56" customHeight="1">
       <c r="A7" s="15" t="n"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>W1–W2</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>10/23</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Navy</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>三套 UI／UX 設計方向</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>快活、政協青年聯會、AI Buddy 各一份設計規範（顏色、字體、圖示、按鈕）和主要頁面線框；快活和政協青年聯會的方向經客戶確認（AI Buddy 可以晚一點）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>W2–W4</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>11/6</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Navy → Jacky</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>快活、政協青年聯會的頁面設計稿</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>配網、綁定、首頁、對話、記憶、設定、語言等頁面的設計稿和切圖交給 Jacky，可以直接做進網頁；政協青年聯會版只換顏色、logo、插圖；客戶確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
           <t>W2–W5</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>11/13</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Navy；Jacky 放進系統</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>角色和內容</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>快活和政協青年聯會每個角色都有人設、說話風格、開場白、聲線和角色圖；每個角色試聽 20 句，客戶確認</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="4" t="inlineStr">
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="16" t="n"/>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>W6–W7</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Navy → Jacky</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>提交 App 圖</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>兩個 App 的圖示、啟動畫面、商店截圖和宣傳圖，按蘋果和 Google 的尺寸交給 Jacky</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="88" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="11" ht="88" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>網頁</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>W1–W3</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>10/30</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>統一開發一套網頁，三套外觀；App 內登入、刪除帳號</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>同一套程式碼按設定切換三套外觀（快活、政協青年聯會、AI Buddy）：顏色、字體、logo、圖示、文案；共用元件裡沒有寫死的品牌；加一套外觀不用改程式；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="15" t="n"/>
-      <c r="B10" s="4" t="inlineStr">
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>W3–W4</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>快活網頁核心：配網、綁定、角色、對話、設定</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>iPhone 和 Android 上 10 分鐘內完成藍牙配網和綁定；選角色、對話、改設定、解綁都正常</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="56" customHeight="1">
-      <c r="A11" s="15" t="n"/>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="13" ht="56" customHeight="1">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>W4–W6</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>快活的功能開關；政協青年聯會套用外觀</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>同一套網頁裡打開快活的功能：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）；政協青年聯會版用同一套成人版流程，只換外觀和角色</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="56" customHeight="1">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="4" t="inlineStr">
+    <row r="14" ht="56" customHeight="1">
+      <c r="A14" s="16" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>功能凍結</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>兩個品牌全流程通過：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁，iOS 和 Android 各至少兩款手機；Wi-Fi 密碼錯、玩具已被綁定、斷網時都有清楚提示</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="72" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>App 殼與上架</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>W1–W2</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>10/23</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Jacky → Neo</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Jacky 交 App 接口參數給 Neo</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>接口文件交給 Neo：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明參數、回傳和錯誤；Neo 確認看得懂、可以開發；兩個 App 的名稱、圖示、bundle id 定好</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="56" customHeight="1">
-      <c r="A14" s="15" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
+    <row r="16" ht="56" customHeight="1">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>W3–W6</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Neo</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>按接口參數開發殼、出測試版</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>兩個 App 的測試版可以安裝（TestFlight、Google 內部測試）；藍牙、登入、推送（玩具上線、低電）可用；連續使用 30 分鐘不閃退</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="56" customHeight="1">
-      <c r="A15" s="15" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>W8–W9</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>12/11</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Neo（客戶提供開發者帳號）</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>提交審核、通過審核</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>11/30 提交，上架資料齊全（截圖、私隱政策、私隱標籤、審核用帳號、玩具示範影片）；12/11 前兩個 App 通過蘋果和 Google 審核</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>W14</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>1/15</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Neo</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>公開上架</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>兩個 App 公開，用戶搜尋得到；App 內看得到客服、常見問題、保修條款</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Tool call</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>W2–W3</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>10/30</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>工具清單和設計</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>1/15 只做兩個工具：調音量、結束對話，寫好觸發說法和回覆方式。其他工具（天氣、日期和節日、快活的賽事資料）上線後經伺服器更新加入</t>
         </is>
       </c>
     </row>
@@ -1757,147 +1753,147 @@
       <c r="A18" s="16" t="n"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>公開上架</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>兩個 App 公開，用戶搜尋得到；App 內看得到客服、常見問題、保修條款</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Tool call</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>W2–W3</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>10/30</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>工具清單和設計</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>1/15 只做兩個工具：調音量、結束對話，寫好觸發說法和回覆方式。其他工具（天氣、日期和節日、快活的賽事資料）上線後經伺服器更新加入</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>W4–W6</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>開發和測試</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>兩個工具各用真實語音觸發 20 次，成功率 ≥ 95%；不相關的話不會誤觸發；首字延遲增加不超過 300 毫秒</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>RAG 知識庫（快活）</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>馬會提供資料；Jacky</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>收資料、入庫流程</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>馬會第一批資料已收到；入庫、版本、審批流程跑通一次</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="56" customHeight="1">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="4" t="inlineStr">
+    <row r="22" ht="56" customHeight="1">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>W5–W8</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>12/4</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>檢索和回答（v1 小版本）</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>v1 只放第一批馬會資料；100 條測試問題答對率 ≥ 80%；知識庫沒有的內容會說不肯定並建議查詢；問貼士、賠率、賽果預測 100% 婉拒</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="16" t="n"/>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>W9–W11</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>12/25</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>馬會審核；Jacky 修改</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>馬會審核 v1</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>馬會書面批准 v1；每一版都有審批記錄；更新知識庫不用重新燒錄玩具</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="56" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>後台管理</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>W3–W6</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>11/20</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>管理功能</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>內容管理員：上載知識庫並送審、發佈角色；超級管理員：看設備最後上線、韌體版本、錯誤，發佈 OTA，解綁和換機；任何管理員都看不到對話內容</t>
         </is>
       </c>
     </row>
@@ -1905,59 +1901,59 @@
       <c r="A23" s="16" t="n"/>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>W6–W8</t>
+          <t>W9–W11</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>12/4</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
+          <t>馬會審核；Jacky 修改</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>馬會審核 v1</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>馬會書面批准 v1；每一版都有審批記錄；更新知識庫不用重新燒錄玩具</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>後台管理</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>W3–W6</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>三個品牌各自一套系統</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>三套各自上線，冒煙測試（登入、對話、OTA 檢查）通過；部署腳本一次跑完三套；一套停機不影響另外兩套</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>W4–W7</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>11/27</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>全體</t>
-        </is>
-      </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>內部測試（20 台、4 週）</t>
+          <t>管理功能</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>每週記錄對話輪數、首字延遲、每台成本、安全事件；第 4 週出測試報告</t>
+          <t>內容管理員：上載知識庫並送審、發佈角色；超級管理員：看設備最後上線、韌體版本、錯誤，發佈 OTA，解綁和換機；任何管理員都看不到對話內容</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1961,7 @@
       <c r="A25" s="16" t="n"/>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>W7–W8</t>
+          <t>W6–W8</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -1980,44 +1976,44 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>系統測試</t>
+          <t>三個品牌各自一套系統</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>全流程測試通過；按 3,000 台規模壓測（150–300 個同時對話）通過；安全測試通過；嚴重問題 0 個</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="56" customHeight="1">
+          <t>三套各自上線，冒煙測試（登入、對話、OTA 檢查）通過；部署腳本一次跑完三套；一套停機不影響另外兩套</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>測試</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>W9–W10</t>
+          <t>W4–W7</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>12/18</t>
+          <t>11/27</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>馬會、政協青年聯會；Jacky</t>
+          <t>全體</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>客戶 UAT（用試產機和正式版 App）</t>
+          <t>內部測試（20 台、4 週）</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>按 UAT 清單逐項測完；馬會、政協青年聯會書面簽收；嚴重問題 0 個，其他問題都有處理日期；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
+          <t>每週記錄對話輪數、首字延遲、每台成本、安全事件；第 4 週出測試報告</t>
         </is>
       </c>
     </row>
@@ -2025,25 +2021,85 @@
       <c r="A27" s="16" t="n"/>
       <c r="B27" s="4" t="inlineStr">
         <is>
+          <t>W7–W8</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>12/4</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>系統測試</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>全流程測試通過；按 3,000 台規模壓測（150–300 個同時對話）通過；安全測試通過；嚴重問題 0 個</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>W9–W10</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>馬會、政協青年聯會；Jacky</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>客戶 UAT（用試產機和正式版 App）</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>按 UAT 清單逐項測完；馬會、政協青年聯會書面簽收；嚴重問題 0 個，其他問題都有處理日期；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="16" t="n"/>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>上線前最後確認</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>UAT 遺留問題全部處理；正式環境凍結，只修 bug；監控和告警正常</t>
         </is>
@@ -2052,15 +2108,15 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A19:A20"/>
     <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A28:A29"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A5:A10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Move work off Jacky and make the firmware deadline visible.
Jacky keeps firmware, architecture, security and integration. Navy also
curates the HKJC data and writes the RAG test set, drafts the character
prompts, and designs the packaging and manual. Neo also runs the phone
testing and the whole store process. A to-be-named coordinator takes the
factory, Spotpear, test lab, client and customer-service follow-ups, and
a third-party inspector does the mid and final inspections.

The software sheet gains a firmware workstream: Bluetooth setup (10/30),
partitions and encryption (11/13), per-brand server URL (11/13), factory
mode and station (11/27), and the image handed to Spotpear on 11/27.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>中期驗貨（12/25–26 香港假期）</t>
+          <t>第三方驗貨公司中期驗貨（12/25–26 香港假期）</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>尾期驗貨；客戶確認 App 公開日期</t>
+          <t>第三方驗貨公司尾期驗貨；客戶確認 App 公開日期</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1227,7 +1227,7 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="10" t="n"/>
     </row>
-    <row r="26" ht="40" customHeight="1">
+    <row r="26" ht="56" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>統籌時間表，對接玩具廠、電路板供應商和客戶；統一開發一套網頁、三套外觀（把 Navy 的設計圖做進 App 畫面）、後台、語音系統、韌體、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；負責測試和 UAT</t>
+          <t>定技術方向；開發韌體（藍牙配網、加密、按品牌連線、出廠工位）、一套網頁三套外觀、後台、語音系統、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；系統測試。與 Claude 協作，雲端的獨立工作可以開多個 session 並行做</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
@@ -1262,14 +1262,14 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>IP 造型設計（政協青年聯會版等），跟進打樣外觀到簽樣；三套 UI／UX 設計；角色和內容（人設、說話風格、開場白、聲線、角色圖）；App 設計圖、圖示、啟動畫面和商店截圖，全部交給 Jacky</t>
+          <t>IP 造型設計（政協青年聯會版等），跟進打樣外觀到簽樣；三套 UI／UX 設計；角色和內容（人設、開場白、聲線、角色圖、提示語初稿）；整理馬會資料、寫 RAG 測試問題；包裝和說明書；App 設計圖、圖示、商店截圖交給 Jacky</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="10" t="n"/>
     </row>
-    <row r="28" ht="40" customHeight="1">
+    <row r="28" ht="56" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Neo</t>
@@ -1278,29 +1278,52 @@
       <c r="B28" s="10" t="n"/>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>App 殼</t>
+          <t>App 殼和上架</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>按 Jacky 給的接口參數，開發 iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；出測試版，提交蘋果和 Google 審核並上架</t>
+          <t>按 Jacky 給的接口參數開發 iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；手機端測試（iOS、Android 各兩款）；整個上架流程，包括跟進客戶開開發者帳號、私隱標籤、審核溝通；UAT 時的手機支援；如熟 Next.js，分擔部分網頁頁面</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
       <c r="G28" s="10" t="n"/>
     </row>
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>對接人（待定）</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>對接和行政</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>建議由老闆或行政／採購同事擔任：跟進玩具廠、Spotpear 的報價、落單、交期和物流；檢測所送檢；安排第三方驗貨公司做中期和尾期驗貨；跟客戶要資料、簽樣、約 UAT；找律師起草私隱政策；內部測試機的分發和回饋；客服聯絡、常見問題、保修條款</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="10" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="D26:G26"/>
+    <mergeCell ref="A29:B29"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="D25:G25"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="D29:G29"/>
     <mergeCell ref="D27:G27"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="D28:G28"/>
@@ -1316,7 +1339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1489,7 +1512,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="15" t="n"/>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -1508,100 +1531,100 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>角色和內容</t>
+          <t>角色和內容（含提示語初稿）</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>快活和政協青年聯會每個角色都有人設、說話風格、開場白、聲線和角色圖；每個角色試聽 20 句，客戶確認</t>
+          <t>快活和政協青年聯會每個角色都有人設、說話風格、開場白、聲線、角色圖，以及提示語初稿（說話規則、禁止話題）；每個角色試聽 20 句，客戶確認</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="16" t="n"/>
+      <c r="A10" s="15" t="n"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>W5–W6</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Navy → 玩具廠</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>包裝和說明書</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>彩盒、說明書（含配網步驟）、App 下載 QR 碼的設計稿交玩具廠打樣；商店描述文字交 Neo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="16" t="n"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
           <t>W6–W7</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Navy → Jacky</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>提交 App 圖</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>兩個 App 的圖示、啟動畫面、商店截圖和宣傳圖，按蘋果和 Google 的尺寸交給 Jacky</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="88" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>網頁</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>W1–W3</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
+    <row r="12" ht="56" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>韌體</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>W2–W3</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>10/30</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>統一開發一套網頁，三套外觀；App 內登入、刪除帳號</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>同一套程式碼按設定切換三套外觀（快活、政協青年聯會、AI Buddy）：顏色、字體、logo、圖示、文案；共用元件裡沒有寫死的品牌；加一套外觀不用改程式；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="15" t="n"/>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>W3–W4</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>11/6</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>快活網頁核心：配網、綁定、角色、對話、設定</t>
+          <t>藍牙配網韌體</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>iPhone 和 Android 上 10 分鐘內完成藍牙配網和綁定；選角色、對話、改設定、解綁都正常</t>
+          <t>廣播帶品牌、回傳 Wi-Fi 清單、收密碼和綁定票、配網後釋放藍牙記憶體；手機 10 分鐘內完成配網和綁定；對話中最低可用記憶體不比現在差</t>
         </is>
       </c>
     </row>
@@ -1609,216 +1632,212 @@
       <c r="A13" s="15" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>W2–W5</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>分區表和加密</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>分區表凍結（加大 app 分區、加品牌資源分區）；一片測試板驗證 Secure Boot 和 Flash 加密：未簽名映像 OTA 被拒，讀出的 flash 是密文</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>W4–W5</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>按品牌連線</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>伺服器網址改為從出廠設定讀取；兩片板寫入不同品牌，各自連上自己那套系統；清空設定後不連任何正式伺服器</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>W5–W7</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>11/27</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>出廠模式和工位腳本</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>經序列埠寫入密鑰、品牌、款式，自檢，再登記到該品牌的系統；連續 10 台通過，混入壞板能攔下</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>11/27</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>出廠韌體定版，交 Spotpear</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>包含以上四項；Spotpear 試燒 10 片，我方驗證通過；記錄版本號。之後只能經 OTA 更新 app 部分</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="88" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>網頁</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>W1–W3</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>10/30</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>統一開發一套網頁，三套外觀；App 內登入、刪除帳號</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>同一套程式碼按設定切換三套外觀（快活、政協青年聯會、AI Buddy）：顏色、字體、logo、圖示、文案；共用元件裡沒有寫死的品牌；加一套外觀不用改程式；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>W3–W4</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>11/6</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>快活網頁核心：配網、綁定、角色、對話、設定</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>iPhone 和 Android 上 10 分鐘內完成藍牙配網和綁定；選角色、對話、改設定、解綁都正常</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>W4–W6</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>快活的功能開關；政協青年聯會套用外觀</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>同一套網頁裡打開快活的功能：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）；政協青年聯會版用同一套成人版流程，只換外觀和角色</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="56" customHeight="1">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>11/27</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>功能凍結</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>兩個品牌全流程通過：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁，iOS 和 Android 各至少兩款手機；Wi-Fi 密碼錯、玩具已被綁定、斷網時都有清楚提示</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="72" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>App 殼與上架</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>W1–W2</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>10/23</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Jacky → Neo</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Jacky 交 App 接口參數給 Neo</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>接口文件交給 Neo：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明參數、回傳和錯誤；Neo 確認看得懂、可以開發；兩個 App 的名稱、圖示、bundle id 定好</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="56" customHeight="1">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>W3–W6</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>11/20</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Neo</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>按接口參數開發殼、出測試版</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>兩個 App 的測試版可以安裝（TestFlight、Google 內部測試）；藍牙、登入、推送（玩具上線、低電）可用；連續使用 30 分鐘不閃退</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="15" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>W8–W9</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>12/11</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Neo（客戶提供開發者帳號）</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>提交審核、通過審核</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>11/30 提交，上架資料齊全（截圖、私隱政策、私隱標籤、審核用帳號、玩具示範影片）；12/11 前兩個 App 通過蘋果和 Google 審核</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="16" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>W14</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>1/15</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Neo</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>公開上架</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>兩個 App 公開，用戶搜尋得到；App 內看得到客服、常見問題、保修條款</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="56" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Tool call</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>W2–W3</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>10/30</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>工具清單和設計</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>1/15 只做兩個工具：調音量、結束對話，寫好觸發說法和回覆方式。其他工具（天氣、日期和節日、快活的賽事資料）上線後經伺服器更新加入</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
+    <row r="20" ht="56" customHeight="1">
       <c r="A20" s="16" t="n"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>W4–W6</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>11/27</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1828,44 +1847,44 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>開發和測試</t>
+          <t>功能凍結</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>兩個工具各用真實語音觸發 20 次，成功率 ≥ 95%；不相關的話不會誤觸發；首字延遲增加不超過 300 毫秒</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1">
+          <t>兩個品牌全流程通過：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁，iOS 和 Android 各至少兩款手機；Wi-Fi 密碼錯、玩具已被綁定、斷網時都有清楚提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>App 殼與上架</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W1–W2</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>11/6</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>馬會提供資料；Jacky</t>
+          <t>Jacky → Neo</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>收資料、入庫流程</t>
+          <t>Jacky 交 App 接口參數給 Neo</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>馬會第一批資料已收到；入庫、版本、審批流程跑通一次</t>
+          <t>接口文件交給 Neo：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明參數、回傳和錯誤；Neo 確認看得懂、可以開發；兩個 App 的名稱、圖示、bundle id 定好</t>
         </is>
       </c>
     </row>
@@ -1873,207 +1892,203 @@
       <c r="A22" s="15" t="n"/>
       <c r="B22" s="4" t="inlineStr">
         <is>
+          <t>W3–W6</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>按接口參數開發殼、出測試版</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>兩個 App 的測試版可以安裝（TestFlight、Google 內部測試）；藍牙、登入、推送（玩具上線、低電）可用；連續使用 30 分鐘不閃退</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="56" customHeight="1">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>W8–W9</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>12/11</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Neo（跟進客戶開帳號、上架資料）</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>提交審核、通過審核</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>11/30 提交，上架資料齊全（截圖、私隱政策、私隱標籤、審核用帳號、玩具示範影片）；12/11 前兩個 App 通過蘋果和 Google 審核</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="16" t="n"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>公開上架</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>兩個 App 公開，用戶搜尋得到；App 內看得到客服、常見問題、保修條款</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="56" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Tool call</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>W2–W3</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>10/30</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>工具清單和設計</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>1/15 只做兩個工具：調音量、結束對話，寫好觸發說法和回覆方式。其他工具（天氣、日期和節日、快活的賽事資料）上線後經伺服器更新加入</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>W4–W6</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>開發和測試</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>兩個工具各用真實語音觸發 20 次，成功率 ≥ 95%；不相關的話不會誤觸發；首字延遲增加不超過 300 毫秒</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>RAG 知識庫（快活）</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>11/6</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>馬會提供資料；Navy 整理；Jacky 入庫</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>收資料、整理、入庫</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>馬會第一批資料已收到；Navy 整理成問答，並寫好 100 條測試問題和標準答案；入庫、版本、審批流程跑通一次</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="15" t="n"/>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
           <t>W5–W8</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>12/4</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>檢索和回答（v1 小版本）</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>v1 只放第一批馬會資料；100 條測試問題答對率 ≥ 80%；知識庫沒有的內容會說不肯定並建議查詢；問貼士、賠率、賽果預測 100% 婉拒</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="16" t="n"/>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>W9–W11</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>12/25</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>馬會審核；Jacky 修改</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>馬會審核 v1</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>馬會書面批准 v1；每一版都有審批記錄；更新知識庫不用重新燒錄玩具</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="56" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>後台管理</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>W3–W6</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>11/20</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>管理功能</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>內容管理員：上載知識庫並送審、發佈角色；超級管理員：看設備最後上線、韌體版本、錯誤，發佈 OTA，解綁和換機；任何管理員都看不到對話內容</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="16" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>W6–W8</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>12/4</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>三個品牌各自一套系統</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>三套各自上線，冒煙測試（登入、對話、OTA 檢查）通過；部署腳本一次跑完三套；一套停機不影響另外兩套</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>W4–W7</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>11/27</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>全體</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>內部測試（20 台、4 週）</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>每週記錄對話輪數、首字延遲、每台成本、安全事件；第 4 週出測試報告</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="16" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>W7–W8</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>12/4</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>系統測試</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>全流程測試通過；按 3,000 台規模壓測（150–300 個同時對話）通過；安全測試通過；嚴重問題 0 個</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="56" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>W9–W10</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>12/18</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>馬會、政協青年聯會；Jacky</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>客戶 UAT（用試產機和正式版 App）</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>按 UAT 清單逐項測完；馬會、政協青年聯會書面簽收；嚴重問題 0 個，其他問題都有處理日期；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
         </is>
       </c>
     </row>
@@ -2081,42 +2096,223 @@
       <c r="A29" s="16" t="n"/>
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>W9–W11</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>12/25</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>馬會審核；Jacky 修改</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>馬會審核 v1</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>馬會書面批准 v1；每一版都有審批記錄；更新知識庫不用重新燒錄玩具</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="56" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>後台管理</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>W3–W6</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>管理功能</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>內容管理員：上載知識庫並送審、發佈角色；超級管理員：看設備最後上線、韌體版本、錯誤，發佈 OTA，解綁和換機；任何管理員都看不到對話內容</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="16" t="n"/>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>W6–W8</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>12/4</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>三個品牌各自一套系統</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>三套各自上線，冒煙測試（登入、對話、OTA 檢查）通過；部署腳本一次跑完三套；一套停機不影響另外兩套</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>W4–W7</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>11/27</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>全體</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>內部測試（20 台、4 週）</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>每週記錄對話輪數、首字延遲、每台成本、安全事件；第 4 週出測試報告</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="56" customHeight="1">
+      <c r="A33" s="16" t="n"/>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>W7–W8</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>12/4</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Jacky；Neo 測手機端</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>系統測試</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>全流程測試通過（Neo 用 iOS、Android 各兩款手機跑）；按 3,000 台規模壓測（150–300 個同時對話）通過；安全測試通過；嚴重問題 0 個</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="56" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>W9–W10</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>對接人約客戶；Jacky、Neo 支援</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>客戶 UAT（用試產機和正式版 App）</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>按 UAT 清單逐項測完；馬會、政協青年聯會書面簽收；嚴重問題 0 個，其他問題都有處理日期；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="16" t="n"/>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Jacky</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>上線前最後確認</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>UAT 遺留問題全部處理；正式環境凍結，只修 bug；監控和告警正常</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A5:A10"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A5:A11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Drop the Claude sentence from Jacky's role.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -1227,7 +1227,7 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="10" t="n"/>
     </row>
-    <row r="26" ht="56" customHeight="1">
+    <row r="26" ht="40" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>定技術方向；開發韌體（藍牙配網、加密、按品牌連線、出廠工位）、一套網頁三套外觀、後台、語音系統、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；系統測試。與 Claude 協作，雲端的獨立工作可以開多個 session 並行做</t>
+          <t>定技術方向；開發韌體（藍牙配網、加密、按品牌連線、出廠工位）、一套網頁三套外觀、後台、語音系統、Tool call 和 RAG，部署三套系統；給 Neo App 接口參數；系統測試</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>

</xml_diff>

<commit_message>
Drop the optional web-pages line from Neo's role.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.6.xlsx
@@ -1269,7 +1269,7 @@
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="10" t="n"/>
     </row>
-    <row r="28" ht="56" customHeight="1">
+    <row r="28" ht="40" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Neo</t>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>按 Jacky 給的接口參數開發 iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；手機端測試（iOS、Android 各兩款）；整個上架流程，包括跟進客戶開開發者帳號、私隱標籤、審核溝通；UAT 時的手機支援；如熟 Next.js，分擔部分網頁頁面</t>
+          <t>按 Jacky 給的接口參數開發 iOS 和 Android 原生殼（藍牙配網、原生登入、推送）；手機端測試（iOS、Android 各兩款）；整個上架流程，包括跟進客戶開開發者帳號、私隱標籤、審核溝通；UAT 時的手機支援</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>

</xml_diff>